<commit_message>
Updated code after review. Added new model variants to the GLMs to address residual vs predicted validation plots. Add mblm models to understand which Dipteran families drove changes through time. Added figure panel labels.
</commit_message>
<xml_diff>
--- a/Taxonomy information/EPT_taxa_for_analysis.xlsx
+++ b/Taxonomy information/EPT_taxa_for_analysis.xlsx
@@ -1,21 +1,485 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gamtostyrimai-my.sharepoint.com/personal/nathan_baker_gamtc_lt/Documents/Breitenbach/Breitenbach_2.0/Taxonomy information/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_A6A83CD48F79A8D366075C52F37BD2728ACF431B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B10973C2-455B-4378-87EF-DF67FFA52321}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="151">
+  <si>
+    <t>sp_name</t>
+  </si>
+  <si>
+    <t>family</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>III</t>
+  </si>
+  <si>
+    <t>Overall</t>
+  </si>
+  <si>
+    <t>Adicella filicornis</t>
+  </si>
+  <si>
+    <t>Leptoceridae</t>
+  </si>
+  <si>
+    <t>Adicella reducta</t>
+  </si>
+  <si>
+    <t>Agapetus fuscipes</t>
+  </si>
+  <si>
+    <t>Glossosomatidae</t>
+  </si>
+  <si>
+    <t>Agraylea multipunctata</t>
+  </si>
+  <si>
+    <t>Hydroptilidae</t>
+  </si>
+  <si>
+    <t>Alainites muticus</t>
+  </si>
+  <si>
+    <t>Baetidae</t>
+  </si>
+  <si>
+    <t>Amphinemura standfussi</t>
+  </si>
+  <si>
+    <t>Nemouridae</t>
+  </si>
+  <si>
+    <t>Amphinemura sulcicollis</t>
+  </si>
+  <si>
+    <t>Anabolia nervosa</t>
+  </si>
+  <si>
+    <t>Limnephilidae</t>
+  </si>
+  <si>
+    <t>Annitella obscurata</t>
+  </si>
+  <si>
+    <t>Apatania fimbriata</t>
+  </si>
+  <si>
+    <t>Apataniidae</t>
+  </si>
+  <si>
+    <t>Athripsodes aterrimus</t>
+  </si>
+  <si>
+    <t>Baetis fuscatus</t>
+  </si>
+  <si>
+    <t>Baetis rhodani</t>
+  </si>
+  <si>
+    <t>Baetis scambus</t>
+  </si>
+  <si>
+    <t>Baetis sp.</t>
+  </si>
+  <si>
+    <t>Baetis vernus</t>
+  </si>
+  <si>
+    <t>Beraea pullata</t>
+  </si>
+  <si>
+    <t>Beraeidae</t>
+  </si>
+  <si>
+    <t>Beraeodes minutus</t>
+  </si>
+  <si>
+    <t>Brachycentrus subnubilus</t>
+  </si>
+  <si>
+    <t>Brachycentridae</t>
+  </si>
+  <si>
+    <t>Brachyptera risi</t>
+  </si>
+  <si>
+    <t>Taeniopterygidae</t>
+  </si>
+  <si>
+    <t>Brachyptera seticornis</t>
+  </si>
+  <si>
+    <t>Centroptilum luteolum</t>
+  </si>
+  <si>
+    <t>Ceraclea dissimilis</t>
+  </si>
+  <si>
+    <t>Chaetopteryx villosa</t>
+  </si>
+  <si>
+    <t>Cheumatopsyche lepida</t>
+  </si>
+  <si>
+    <t>Hydropsychidae</t>
+  </si>
+  <si>
+    <t>Crunoecia irrorata</t>
+  </si>
+  <si>
+    <t>Lepidostomatidae</t>
+  </si>
+  <si>
+    <t>Cyrnus trimaculatus</t>
+  </si>
+  <si>
+    <t>Polycentropodidae</t>
+  </si>
+  <si>
+    <t>Diplectrona felix</t>
+  </si>
+  <si>
+    <t>Drusus annulatus</t>
+  </si>
+  <si>
+    <t>Drusus biguttatus</t>
+  </si>
+  <si>
+    <t>Ecdyonurus sp.</t>
+  </si>
+  <si>
+    <t>Heptageniidae</t>
+  </si>
+  <si>
+    <t>Epeorus sp.</t>
+  </si>
+  <si>
+    <t>Ephemera danica</t>
+  </si>
+  <si>
+    <t>Ephemeridae</t>
+  </si>
+  <si>
+    <t>Ephemerella mucronata</t>
+  </si>
+  <si>
+    <t>Ephemerellidae</t>
+  </si>
+  <si>
+    <t>Glossosoma conformis</t>
+  </si>
+  <si>
+    <t>Glyphotaelius pellucidus</t>
+  </si>
+  <si>
+    <t>Grammotaulius nigropunctatus</t>
+  </si>
+  <si>
+    <t>Grammotaulius nitidus</t>
+  </si>
+  <si>
+    <t>Habrophlebia fusca</t>
+  </si>
+  <si>
+    <t>Leptophlebiidae</t>
+  </si>
+  <si>
+    <t>Habrophlebia lauta</t>
+  </si>
+  <si>
+    <t>Halesus digitatus</t>
+  </si>
+  <si>
+    <t>Halesus radiatus</t>
+  </si>
+  <si>
+    <t>Halesus tesselatus</t>
+  </si>
+  <si>
+    <t>Hydropsyche angustipennis</t>
+  </si>
+  <si>
+    <t>Hydropsyche instabilis</t>
+  </si>
+  <si>
+    <t>Hydropsyche pellucidula</t>
+  </si>
+  <si>
+    <t>Hydropsyche saxonica</t>
+  </si>
+  <si>
+    <t>Hydropsyche siltalai</t>
+  </si>
+  <si>
+    <t>Hydropsyche sp.</t>
+  </si>
+  <si>
+    <t>Hydroptila pulchricornis</t>
+  </si>
+  <si>
+    <t>Hydroptila sparsa</t>
+  </si>
+  <si>
+    <t>Isoperla grammatica</t>
+  </si>
+  <si>
+    <t>Perlodidae</t>
+  </si>
+  <si>
+    <t>Isoperla sp.</t>
+  </si>
+  <si>
+    <t>Lasiocephala basalis</t>
+  </si>
+  <si>
+    <t>Leuctra braueri</t>
+  </si>
+  <si>
+    <t>Leuctridae</t>
+  </si>
+  <si>
+    <t>Leuctra digitata</t>
+  </si>
+  <si>
+    <t>Leuctra fusca</t>
+  </si>
+  <si>
+    <t>Leuctra inermis</t>
+  </si>
+  <si>
+    <t>Leuctra nigra</t>
+  </si>
+  <si>
+    <t>Leuctra prima</t>
+  </si>
+  <si>
+    <t>Leuctra sp.</t>
+  </si>
+  <si>
+    <t>Limnephilus auricula</t>
+  </si>
+  <si>
+    <t>Limnephilus bipunctatus</t>
+  </si>
+  <si>
+    <t>Limnephilus centralis</t>
+  </si>
+  <si>
+    <t>Limnephilus extricatus</t>
+  </si>
+  <si>
+    <t>Limnephilus fuscicornis</t>
+  </si>
+  <si>
+    <t>Limnephilus griseus</t>
+  </si>
+  <si>
+    <t>Limnephilus hirsutus</t>
+  </si>
+  <si>
+    <t>Limnephilus ignavus</t>
+  </si>
+  <si>
+    <t>Limnephilus lunatus</t>
+  </si>
+  <si>
+    <t>Limnephilus rhombicus</t>
+  </si>
+  <si>
+    <t>Limnephilus sparsus</t>
+  </si>
+  <si>
+    <t>Lype phaeopa</t>
+  </si>
+  <si>
+    <t>Psychomyiidae</t>
+  </si>
+  <si>
+    <t>Lype reducta</t>
+  </si>
+  <si>
+    <t>Micrasema longulum</t>
+  </si>
+  <si>
+    <t>Mystacides longicornis</t>
+  </si>
+  <si>
+    <t>Nemoura cambrica</t>
+  </si>
+  <si>
+    <t>Nemoura cinerea</t>
+  </si>
+  <si>
+    <t>Nemoura flexuosa</t>
+  </si>
+  <si>
+    <t>Nemoura marginata</t>
+  </si>
+  <si>
+    <t>Nemoura sciurus</t>
+  </si>
+  <si>
+    <t>Nemoura sp.</t>
+  </si>
+  <si>
+    <t>Nemurella pictetii</t>
+  </si>
+  <si>
+    <t>Odontocerum albicorne</t>
+  </si>
+  <si>
+    <t>Odontoceridae</t>
+  </si>
+  <si>
+    <t>Paraleptophlebia submarginata</t>
+  </si>
+  <si>
+    <t>Perlodes dispar</t>
+  </si>
+  <si>
+    <t>Perlodes microcephalus</t>
+  </si>
+  <si>
+    <t>Plectrocnemia conspersa</t>
+  </si>
+  <si>
+    <t>Potamophylax cingulatus</t>
+  </si>
+  <si>
+    <t>Potamophylax latipennis</t>
+  </si>
+  <si>
+    <t>Potamophylax luctuosus</t>
+  </si>
+  <si>
+    <t>Potamophylax nigricornis</t>
+  </si>
+  <si>
+    <t>Protonemura auberti</t>
+  </si>
+  <si>
+    <t>Protonemura intricata</t>
+  </si>
+  <si>
+    <t>Protonemura meyeri</t>
+  </si>
+  <si>
+    <t>Protonemura nitida</t>
+  </si>
+  <si>
+    <t>Psychomyia pusilla</t>
+  </si>
+  <si>
+    <t>Ptilocolepus granulatus</t>
+  </si>
+  <si>
+    <t>Rhithrogena sp.</t>
+  </si>
+  <si>
+    <t>Rhyacophila fasciata</t>
+  </si>
+  <si>
+    <t>Rhyacophilidae</t>
+  </si>
+  <si>
+    <t>Rhyacophila nubila</t>
+  </si>
+  <si>
+    <t>Sericostoma flavicorne</t>
+  </si>
+  <si>
+    <t>Sericostomatidae</t>
+  </si>
+  <si>
+    <t>Sericostoma personatum</t>
+  </si>
+  <si>
+    <t>Serratella ignita</t>
+  </si>
+  <si>
+    <t>Silo pallipes</t>
+  </si>
+  <si>
+    <t>Goeridae</t>
+  </si>
+  <si>
+    <t>Siphonoperla torrentium</t>
+  </si>
+  <si>
+    <t>Chloroperlidae</t>
+  </si>
+  <si>
+    <t>Stenophylax lateralis</t>
+  </si>
+  <si>
+    <t>Stenophylax nycterobius</t>
+  </si>
+  <si>
+    <t>Stenophylax permistus</t>
+  </si>
+  <si>
+    <t>Stenophylax sequax</t>
+  </si>
+  <si>
+    <t>Synagapetus moselyi</t>
+  </si>
+  <si>
+    <t>Tinodes pallidulus</t>
+  </si>
+  <si>
+    <t>Tinodes rostocki</t>
+  </si>
+  <si>
+    <t>Tinodes waeneri</t>
+  </si>
+  <si>
+    <t>Wormaldia occipitalis</t>
+  </si>
+  <si>
+    <t>Philopotamidae</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -63,13 +527,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -107,7 +579,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -141,6 +613,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -175,9 +648,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -350,72 +824,52 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J116"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.54296875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>sp_name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>family</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>III</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Adicella filicornis</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Leptoceridae</t>
-        </is>
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
       </c>
       <c r="C2">
         <v>20</v>
@@ -442,16 +896,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Adicella reducta</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Leptoceridae</t>
-        </is>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
       </c>
       <c r="C3">
         <v>34</v>
@@ -478,16 +928,12 @@
         <v>1589</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Agapetus fuscipes</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Glossosomatidae</t>
-        </is>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
       </c>
       <c r="C4">
         <v>91457</v>
@@ -514,16 +960,12 @@
         <v>275025</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Agraylea multipunctata</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Hydroptilidae</t>
-        </is>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -550,16 +992,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Alainites muticus</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Baetidae</t>
-        </is>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -586,16 +1024,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Amphinemura standfussi</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
       </c>
       <c r="C7">
         <v>3663</v>
@@ -622,16 +1056,12 @@
         <v>14201</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Amphinemura sulcicollis</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -658,16 +1088,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Anabolia nervosa</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -694,16 +1120,12 @@
         <v>54</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Annitella obscurata</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -730,16 +1152,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Apatania fimbriata</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Apataniidae</t>
-        </is>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
       </c>
       <c r="C11">
         <v>5466</v>
@@ -766,16 +1184,12 @@
         <v>27391</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Athripsodes aterrimus</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Leptoceridae</t>
-        </is>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -802,16 +1216,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Baetis fuscatus</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Baetidae</t>
-        </is>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
+        <v>18</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -838,16 +1248,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Baetis rhodani</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Baetidae</t>
-        </is>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>18</v>
       </c>
       <c r="C14">
         <v>3869</v>
@@ -874,16 +1280,12 @@
         <v>144765</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Baetis scambus</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Baetidae</t>
-        </is>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -910,16 +1312,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Baetis sp.</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Baetidae</t>
-        </is>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
+        <v>18</v>
       </c>
       <c r="C16">
         <v>1012</v>
@@ -946,16 +1344,12 @@
         <v>12731</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Baetis vernus</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Baetidae</t>
-        </is>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>18</v>
       </c>
       <c r="C17">
         <v>16517</v>
@@ -982,16 +1376,12 @@
         <v>349522</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Beraea pullata</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Beraeidae</t>
-        </is>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" t="s">
+        <v>34</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -1018,16 +1408,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Beraeodes minutus</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Beraeidae</t>
-        </is>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" t="s">
+        <v>34</v>
       </c>
       <c r="C19">
         <v>3</v>
@@ -1054,16 +1440,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Brachycentrus subnubilus</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Brachycentridae</t>
-        </is>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" t="s">
+        <v>37</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -1090,16 +1472,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Brachyptera risi</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Taeniopterygidae</t>
-        </is>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" t="s">
+        <v>39</v>
       </c>
       <c r="C21">
         <v>2966</v>
@@ -1126,16 +1504,12 @@
         <v>4016</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Brachyptera seticornis</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Taeniopterygidae</t>
-        </is>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" t="s">
+        <v>39</v>
       </c>
       <c r="C22">
         <v>88</v>
@@ -1162,16 +1536,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Centroptilum luteolum</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Baetidae</t>
-        </is>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" t="s">
+        <v>18</v>
       </c>
       <c r="C23">
         <v>31</v>
@@ -1198,16 +1568,12 @@
         <v>5400</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Ceraclea dissimilis</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Leptoceridae</t>
-        </is>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -1234,16 +1600,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Chaetopteryx villosa</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" t="s">
+        <v>23</v>
       </c>
       <c r="C25">
         <v>12343</v>
@@ -1270,16 +1632,12 @@
         <v>42543</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Cheumatopsyche lepida</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Hydropsychidae</t>
-        </is>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" t="s">
+        <v>45</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -1306,16 +1664,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Crunoecia irrorata</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Lepidostomatidae</t>
-        </is>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" t="s">
+        <v>47</v>
       </c>
       <c r="C27">
         <v>2</v>
@@ -1342,16 +1696,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Cyrnus trimaculatus</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Polycentropodidae</t>
-        </is>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" t="s">
+        <v>49</v>
       </c>
       <c r="C28">
         <v>2</v>
@@ -1378,16 +1728,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Diplectrona felix</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Hydropsychidae</t>
-        </is>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" t="s">
+        <v>45</v>
       </c>
       <c r="C29">
         <v>0</v>
@@ -1414,16 +1760,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Drusus annulatus</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" t="s">
+        <v>23</v>
       </c>
       <c r="C30">
         <v>1897</v>
@@ -1450,16 +1792,12 @@
         <v>6797</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Drusus biguttatus</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" t="s">
+        <v>23</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -1486,16 +1824,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Ecdyonurus sp.</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Heptageniidae</t>
-        </is>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>53</v>
+      </c>
+      <c r="B32" t="s">
+        <v>54</v>
       </c>
       <c r="C32">
         <v>4</v>
@@ -1522,16 +1856,12 @@
         <v>533</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Epeorus sp.</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Heptageniidae</t>
-        </is>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" t="s">
+        <v>54</v>
       </c>
       <c r="C33">
         <v>67</v>
@@ -1558,16 +1888,12 @@
         <v>383</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Ephemera danica</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Ephemeridae</t>
-        </is>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" t="s">
+        <v>57</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -1594,16 +1920,12 @@
         <v>39</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Ephemerella mucronata</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Ephemerellidae</t>
-        </is>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>58</v>
+      </c>
+      <c r="B35" t="s">
+        <v>59</v>
       </c>
       <c r="C35">
         <v>9</v>
@@ -1630,16 +1952,12 @@
         <v>13755</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Glossosoma conformis</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Glossosomatidae</t>
-        </is>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" t="s">
+        <v>14</v>
       </c>
       <c r="C36">
         <v>0</v>
@@ -1666,16 +1984,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Glyphotaelius pellucidus</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" t="s">
+        <v>23</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -1702,16 +2016,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Grammotaulius nigropunctatus</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" t="s">
+        <v>23</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -1738,16 +2048,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Grammotaulius nitidus</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B39" t="s">
+        <v>23</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -1774,16 +2080,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Habrophlebia fusca</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Leptophlebiidae</t>
-        </is>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>64</v>
+      </c>
+      <c r="B40" t="s">
+        <v>65</v>
       </c>
       <c r="C40">
         <v>11</v>
@@ -1810,16 +2112,12 @@
         <v>155</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Habrophlebia lauta</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Leptophlebiidae</t>
-        </is>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>66</v>
+      </c>
+      <c r="B41" t="s">
+        <v>65</v>
       </c>
       <c r="C41">
         <v>3</v>
@@ -1846,16 +2144,12 @@
         <v>256</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Halesus digitatus</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42" t="s">
+        <v>23</v>
       </c>
       <c r="C42">
         <v>43</v>
@@ -1882,16 +2176,12 @@
         <v>449</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Halesus radiatus</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>68</v>
+      </c>
+      <c r="B43" t="s">
+        <v>23</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -1918,16 +2208,12 @@
         <v>105</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Halesus tesselatus</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>69</v>
+      </c>
+      <c r="B44" t="s">
+        <v>23</v>
       </c>
       <c r="C44">
         <v>0</v>
@@ -1954,16 +2240,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Hydropsyche angustipennis</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Hydropsychidae</t>
-        </is>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>70</v>
+      </c>
+      <c r="B45" t="s">
+        <v>45</v>
       </c>
       <c r="C45">
         <v>0</v>
@@ -1990,16 +2272,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Hydropsyche instabilis</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Hydropsychidae</t>
-        </is>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>71</v>
+      </c>
+      <c r="B46" t="s">
+        <v>45</v>
       </c>
       <c r="C46">
         <v>7</v>
@@ -2026,16 +2304,12 @@
         <v>1968</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Hydropsyche pellucidula</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Hydropsychidae</t>
-        </is>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>72</v>
+      </c>
+      <c r="B47" t="s">
+        <v>45</v>
       </c>
       <c r="C47">
         <v>0</v>
@@ -2062,16 +2336,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Hydropsyche saxonica</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Hydropsychidae</t>
-        </is>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48" t="s">
+        <v>45</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -2098,16 +2368,12 @@
         <v>755</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Hydropsyche siltalai</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Hydropsychidae</t>
-        </is>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B49" t="s">
+        <v>45</v>
       </c>
       <c r="C49">
         <v>3</v>
@@ -2134,16 +2400,12 @@
         <v>122</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Hydropsyche sp.</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Hydropsychidae</t>
-        </is>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>75</v>
+      </c>
+      <c r="B50" t="s">
+        <v>45</v>
       </c>
       <c r="C50">
         <v>0</v>
@@ -2170,16 +2432,12 @@
         <v>615</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Hydroptila pulchricornis</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Hydroptilidae</t>
-        </is>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>76</v>
+      </c>
+      <c r="B51" t="s">
+        <v>16</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -2206,16 +2464,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Hydroptila sparsa</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Hydroptilidae</t>
-        </is>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>77</v>
+      </c>
+      <c r="B52" t="s">
+        <v>16</v>
       </c>
       <c r="C52">
         <v>0</v>
@@ -2242,16 +2496,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Isoperla grammatica</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Perlodidae</t>
-        </is>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>78</v>
+      </c>
+      <c r="B53" t="s">
+        <v>79</v>
       </c>
       <c r="C53">
         <v>3</v>
@@ -2278,16 +2528,12 @@
         <v>90</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Isoperla sp.</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Perlodidae</t>
-        </is>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54" t="s">
+        <v>79</v>
       </c>
       <c r="C54">
         <v>1242</v>
@@ -2314,16 +2560,12 @@
         <v>10124</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Lasiocephala basalis</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Lepidostomatidae</t>
-        </is>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>81</v>
+      </c>
+      <c r="B55" t="s">
+        <v>47</v>
       </c>
       <c r="C55">
         <v>2</v>
@@ -2350,16 +2592,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Leuctra braueri</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Leuctridae</t>
-        </is>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
+      <c r="B56" t="s">
+        <v>83</v>
       </c>
       <c r="C56">
         <v>0</v>
@@ -2386,16 +2624,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Leuctra digitata</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Leuctridae</t>
-        </is>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>84</v>
+      </c>
+      <c r="B57" t="s">
+        <v>83</v>
       </c>
       <c r="C57">
         <v>1549</v>
@@ -2422,16 +2656,12 @@
         <v>72418</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Leuctra fusca</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Leuctridae</t>
-        </is>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>85</v>
+      </c>
+      <c r="B58" t="s">
+        <v>83</v>
       </c>
       <c r="C58">
         <v>0</v>
@@ -2458,16 +2688,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Leuctra inermis</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Leuctridae</t>
-        </is>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>86</v>
+      </c>
+      <c r="B59" t="s">
+        <v>83</v>
       </c>
       <c r="C59">
         <v>4</v>
@@ -2494,16 +2720,12 @@
         <v>61</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Leuctra nigra</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Leuctridae</t>
-        </is>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>87</v>
+      </c>
+      <c r="B60" t="s">
+        <v>83</v>
       </c>
       <c r="C60">
         <v>10221</v>
@@ -2530,16 +2752,12 @@
         <v>161811</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Leuctra prima</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Leuctridae</t>
-        </is>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>88</v>
+      </c>
+      <c r="B61" t="s">
+        <v>83</v>
       </c>
       <c r="C61">
         <v>9070</v>
@@ -2566,16 +2784,12 @@
         <v>37863</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Leuctra sp.</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Leuctridae</t>
-        </is>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>89</v>
+      </c>
+      <c r="B62" t="s">
+        <v>83</v>
       </c>
       <c r="C62">
         <v>14</v>
@@ -2602,16 +2816,12 @@
         <v>225</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Limnephilus auricula</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>90</v>
+      </c>
+      <c r="B63" t="s">
+        <v>23</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -2638,16 +2848,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Limnephilus bipunctatus</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64" t="s">
+        <v>23</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -2674,16 +2880,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Limnephilus centralis</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>92</v>
+      </c>
+      <c r="B65" t="s">
+        <v>23</v>
       </c>
       <c r="C65">
         <v>11</v>
@@ -2710,16 +2912,12 @@
         <v>91</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Limnephilus extricatus</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66" t="s">
+        <v>23</v>
       </c>
       <c r="C66">
         <v>0</v>
@@ -2746,16 +2944,12 @@
         <v>81</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Limnephilus fuscicornis</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67" t="s">
+        <v>23</v>
       </c>
       <c r="C67">
         <v>0</v>
@@ -2782,16 +2976,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Limnephilus griseus</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>95</v>
+      </c>
+      <c r="B68" t="s">
+        <v>23</v>
       </c>
       <c r="C68">
         <v>0</v>
@@ -2818,16 +3008,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Limnephilus hirsutus</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69" t="s">
+        <v>23</v>
       </c>
       <c r="C69">
         <v>0</v>
@@ -2854,16 +3040,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Limnephilus ignavus</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>97</v>
+      </c>
+      <c r="B70" t="s">
+        <v>23</v>
       </c>
       <c r="C70">
         <v>0</v>
@@ -2890,16 +3072,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Limnephilus lunatus</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>98</v>
+      </c>
+      <c r="B71" t="s">
+        <v>23</v>
       </c>
       <c r="C71">
         <v>0</v>
@@ -2926,16 +3104,12 @@
         <v>48</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Limnephilus rhombicus</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>99</v>
+      </c>
+      <c r="B72" t="s">
+        <v>23</v>
       </c>
       <c r="C72">
         <v>6</v>
@@ -2962,16 +3136,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Limnephilus sparsus</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>100</v>
+      </c>
+      <c r="B73" t="s">
+        <v>23</v>
       </c>
       <c r="C73">
         <v>18</v>
@@ -2998,16 +3168,12 @@
         <v>523</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Lype phaeopa</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Psychomyiidae</t>
-        </is>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>101</v>
+      </c>
+      <c r="B74" t="s">
+        <v>102</v>
       </c>
       <c r="C74">
         <v>0</v>
@@ -3034,16 +3200,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Lype reducta</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Psychomyiidae</t>
-        </is>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>103</v>
+      </c>
+      <c r="B75" t="s">
+        <v>102</v>
       </c>
       <c r="C75">
         <v>1</v>
@@ -3070,16 +3232,12 @@
         <v>675</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Micrasema longulum</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Brachycentridae</t>
-        </is>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76" t="s">
+        <v>37</v>
       </c>
       <c r="C76">
         <v>7</v>
@@ -3106,16 +3264,12 @@
         <v>651</v>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Mystacides longicornis</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Leptoceridae</t>
-        </is>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B77" t="s">
+        <v>11</v>
       </c>
       <c r="C77">
         <v>1</v>
@@ -3142,16 +3296,12 @@
         <v>62</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Nemoura cambrica</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>106</v>
+      </c>
+      <c r="B78" t="s">
+        <v>20</v>
       </c>
       <c r="C78">
         <v>3381</v>
@@ -3178,16 +3328,12 @@
         <v>22821</v>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Nemoura cinerea</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>107</v>
+      </c>
+      <c r="B79" t="s">
+        <v>20</v>
       </c>
       <c r="C79">
         <v>271</v>
@@ -3214,16 +3360,12 @@
         <v>1265</v>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Nemoura flexuosa</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80" t="s">
+        <v>20</v>
       </c>
       <c r="C80">
         <v>280</v>
@@ -3250,16 +3392,12 @@
         <v>8929</v>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Nemoura marginata</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81" t="s">
+        <v>20</v>
       </c>
       <c r="C81">
         <v>2089</v>
@@ -3286,16 +3424,12 @@
         <v>6030</v>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Nemoura sciurus</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82" t="s">
+        <v>20</v>
       </c>
       <c r="C82">
         <v>0</v>
@@ -3322,16 +3456,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Nemoura sp.</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>111</v>
+      </c>
+      <c r="B83" t="s">
+        <v>20</v>
       </c>
       <c r="C83">
         <v>1712</v>
@@ -3358,16 +3488,12 @@
         <v>12058</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>Nemurella pictetii</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>112</v>
+      </c>
+      <c r="B84" t="s">
+        <v>20</v>
       </c>
       <c r="C84">
         <v>5173</v>
@@ -3394,16 +3520,12 @@
         <v>17137</v>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>Odontocerum albicorne</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>Odontoceridae</t>
-        </is>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>113</v>
+      </c>
+      <c r="B85" t="s">
+        <v>114</v>
       </c>
       <c r="C85">
         <v>0</v>
@@ -3430,16 +3552,12 @@
         <v>280</v>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>Paraleptophlebia submarginata</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Leptophlebiidae</t>
-        </is>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>115</v>
+      </c>
+      <c r="B86" t="s">
+        <v>65</v>
       </c>
       <c r="C86">
         <v>86</v>
@@ -3466,16 +3584,12 @@
         <v>9503</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>Perlodes dispar</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Perlodidae</t>
-        </is>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87" t="s">
+        <v>79</v>
       </c>
       <c r="C87">
         <v>0</v>
@@ -3502,16 +3616,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Perlodes microcephalus</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Perlodidae</t>
-        </is>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>117</v>
+      </c>
+      <c r="B88" t="s">
+        <v>79</v>
       </c>
       <c r="C88">
         <v>1</v>
@@ -3538,16 +3648,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>Plectrocnemia conspersa</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Polycentropodidae</t>
-        </is>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>118</v>
+      </c>
+      <c r="B89" t="s">
+        <v>49</v>
       </c>
       <c r="C89">
         <v>926</v>
@@ -3574,16 +3680,12 @@
         <v>6070</v>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>Potamophylax cingulatus</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>119</v>
+      </c>
+      <c r="B90" t="s">
+        <v>23</v>
       </c>
       <c r="C90">
         <v>632</v>
@@ -3610,16 +3712,12 @@
         <v>1676</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>Potamophylax latipennis</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>120</v>
+      </c>
+      <c r="B91" t="s">
+        <v>23</v>
       </c>
       <c r="C91">
         <v>0</v>
@@ -3646,16 +3744,12 @@
         <v>196</v>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>Potamophylax luctuosus</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>121</v>
+      </c>
+      <c r="B92" t="s">
+        <v>23</v>
       </c>
       <c r="C92">
         <v>21</v>
@@ -3682,16 +3776,12 @@
         <v>1206</v>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>Potamophylax nigricornis</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93" t="s">
+        <v>23</v>
       </c>
       <c r="C93">
         <v>17</v>
@@ -3718,16 +3808,12 @@
         <v>26</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>Protonemura auberti</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>123</v>
+      </c>
+      <c r="B94" t="s">
+        <v>20</v>
       </c>
       <c r="C94">
         <v>10579</v>
@@ -3754,16 +3840,12 @@
         <v>30147</v>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>Protonemura intricata</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>124</v>
+      </c>
+      <c r="B95" t="s">
+        <v>20</v>
       </c>
       <c r="C95">
         <v>9512</v>
@@ -3790,16 +3872,12 @@
         <v>109787</v>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>Protonemura meyeri</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>125</v>
+      </c>
+      <c r="B96" t="s">
+        <v>20</v>
       </c>
       <c r="C96">
         <v>2158</v>
@@ -3826,16 +3904,12 @@
         <v>12062</v>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>Protonemura nitida</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Nemouridae</t>
-        </is>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>126</v>
+      </c>
+      <c r="B97" t="s">
+        <v>20</v>
       </c>
       <c r="C97">
         <v>9</v>
@@ -3862,16 +3936,12 @@
         <v>490</v>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>Psychomyia pusilla</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Psychomyiidae</t>
-        </is>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>127</v>
+      </c>
+      <c r="B98" t="s">
+        <v>102</v>
       </c>
       <c r="C98">
         <v>1</v>
@@ -3898,16 +3968,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>Ptilocolepus granulatus</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Hydroptilidae</t>
-        </is>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99" t="s">
+        <v>16</v>
       </c>
       <c r="C99">
         <v>1</v>
@@ -3934,16 +4000,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>Rhithrogena sp.</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>Heptageniidae</t>
-        </is>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>129</v>
+      </c>
+      <c r="B100" t="s">
+        <v>54</v>
       </c>
       <c r="C100">
         <v>0</v>
@@ -3970,16 +4032,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>Rhyacophila fasciata</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Rhyacophilidae</t>
-        </is>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101" t="s">
+        <v>131</v>
       </c>
       <c r="C101">
         <v>488</v>
@@ -4006,16 +4064,12 @@
         <v>7534</v>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>Rhyacophila nubila</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>Rhyacophilidae</t>
-        </is>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>132</v>
+      </c>
+      <c r="B102" t="s">
+        <v>131</v>
       </c>
       <c r="C102">
         <v>1</v>
@@ -4042,16 +4096,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Sericostoma flavicorne</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>Sericostomatidae</t>
-        </is>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>133</v>
+      </c>
+      <c r="B103" t="s">
+        <v>134</v>
       </c>
       <c r="C103">
         <v>0</v>
@@ -4078,16 +4128,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>Sericostoma personatum</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Sericostomatidae</t>
-        </is>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>135</v>
+      </c>
+      <c r="B104" t="s">
+        <v>134</v>
       </c>
       <c r="C104">
         <v>1756</v>
@@ -4114,16 +4160,12 @@
         <v>13991</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
-        <is>
-          <t>Serratella ignita</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Ephemerellidae</t>
-        </is>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>136</v>
+      </c>
+      <c r="B105" t="s">
+        <v>59</v>
       </c>
       <c r="C105">
         <v>10</v>
@@ -4150,16 +4192,12 @@
         <v>12392</v>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>Silo pallipes</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>Goeridae</t>
-        </is>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>137</v>
+      </c>
+      <c r="B106" t="s">
+        <v>138</v>
       </c>
       <c r="C106">
         <v>38</v>
@@ -4186,16 +4224,12 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>Siphonoperla torrentium</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Chloroperlidae</t>
-        </is>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>139</v>
+      </c>
+      <c r="B107" t="s">
+        <v>140</v>
       </c>
       <c r="C107">
         <v>2177</v>
@@ -4222,16 +4256,12 @@
         <v>22055</v>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>Stenophylax lateralis</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>141</v>
+      </c>
+      <c r="B108" t="s">
+        <v>23</v>
       </c>
       <c r="C108">
         <v>23</v>
@@ -4258,16 +4288,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>Stenophylax nycterobius</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>142</v>
+      </c>
+      <c r="B109" t="s">
+        <v>23</v>
       </c>
       <c r="C109">
         <v>1</v>
@@ -4294,16 +4320,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>Stenophylax permistus</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>143</v>
+      </c>
+      <c r="B110" t="s">
+        <v>23</v>
       </c>
       <c r="C110">
         <v>5</v>
@@ -4330,16 +4352,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>Stenophylax sequax</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Limnephilidae</t>
-        </is>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
+        <v>144</v>
+      </c>
+      <c r="B111" t="s">
+        <v>23</v>
       </c>
       <c r="C111">
         <v>364</v>
@@ -4366,16 +4384,12 @@
         <v>403</v>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>Synagapetus moselyi</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>Glossosomatidae</t>
-        </is>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>145</v>
+      </c>
+      <c r="B112" t="s">
+        <v>14</v>
       </c>
       <c r="C112">
         <v>1</v>
@@ -4402,16 +4416,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>Tinodes pallidulus</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>Psychomyiidae</t>
-        </is>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>146</v>
+      </c>
+      <c r="B113" t="s">
+        <v>102</v>
       </c>
       <c r="C113">
         <v>0</v>
@@ -4438,16 +4448,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>Tinodes rostocki</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>Psychomyiidae</t>
-        </is>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
+        <v>147</v>
+      </c>
+      <c r="B114" t="s">
+        <v>102</v>
       </c>
       <c r="C114">
         <v>3292</v>
@@ -4474,16 +4480,12 @@
         <v>87560</v>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>Tinodes waeneri</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>Psychomyiidae</t>
-        </is>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
+        <v>148</v>
+      </c>
+      <c r="B115" t="s">
+        <v>102</v>
       </c>
       <c r="C115">
         <v>0</v>
@@ -4510,16 +4512,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Wormaldia occipitalis</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Philopotamidae</t>
-        </is>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>149</v>
+      </c>
+      <c r="B116" t="s">
+        <v>150</v>
       </c>
       <c r="C116">
         <v>2107</v>

</xml_diff>